<commit_message>
Excel Mapping v14.6: Added Shinhan Card template and smart date parsing
</commit_message>
<xml_diff>
--- a/26년1월 이용대금명세서(신용카드).xlsx
+++ b/26년1월 이용대금명세서(신용카드).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\ks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{738D654A-AC23-419B-A517-CB681D11E96E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597B6B1F-08CD-461F-81A1-E5E9A7710C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4095" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{52355010-6A33-4467-A1FA-07BC115C4BA9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52355010-6A33-4467-A1FA-07BC115C4BA9}"/>
   </bookViews>
   <sheets>
     <sheet name="26년1월 이용대금명세서(신용카드)" sheetId="2" r:id="rId1"/>
@@ -865,7 +865,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1043,6 +1043,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1459,7 +1465,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1475,41 +1481,161 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1520,143 +1646,38 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2049,26 +2070,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
+      <c r="A1" s="57" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="11"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="38"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -2080,14 +2101,14 @@
       <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="5" t="s">
+      <c r="E3" s="23"/>
+      <c r="F3" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -2099,133 +2120,133 @@
       <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="7" t="s">
+      <c r="D4" s="24"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="8"/>
+      <c r="G4" s="26"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="22"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="53"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="25"/>
+      <c r="B6" s="49"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="50"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="28"/>
+      <c r="A7" s="54"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="56"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="25"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="50"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="50"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28"/>
+      <c r="A10" s="54"/>
+      <c r="B10" s="55"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="56"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="25"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="50"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="31"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="37"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="39"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="5" t="s">
+      <c r="B14" s="22"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="6"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="23"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="35" t="s">
+      <c r="B15" s="19"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="36"/>
-      <c r="G15" s="37"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="20"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="9" t="s">
+      <c r="B16" s="33"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="11"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="38"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -2237,7 +2258,7 @@
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="41"/>
+      <c r="D17" s="40"/>
       <c r="E17" s="1" t="s">
         <v>38</v>
       </c>
@@ -2249,18 +2270,18 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="32">
+      <c r="B18" s="23"/>
+      <c r="C18" s="10">
         <v>1122842</v>
       </c>
-      <c r="D18" s="41"/>
+      <c r="D18" s="40"/>
       <c r="E18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="12">
         <v>14116</v>
       </c>
       <c r="G18" s="3">
@@ -2277,10 +2298,10 @@
       <c r="C19" s="3">
         <v>0</v>
       </c>
-      <c r="D19" s="41"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="8"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -2292,27 +2313,27 @@
       <c r="C20" s="3">
         <v>0</v>
       </c>
-      <c r="D20" s="41"/>
-      <c r="E20" s="5" t="s">
+      <c r="D20" s="40"/>
+      <c r="E20" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="6"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="23"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="33">
-        <v>0</v>
-      </c>
-      <c r="D21" s="41"/>
-      <c r="E21" s="35" t="s">
+      <c r="B21" s="23"/>
+      <c r="C21" s="11">
+        <v>0</v>
+      </c>
+      <c r="D21" s="40"/>
+      <c r="E21" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="36"/>
-      <c r="G21" s="37"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -2324,12 +2345,12 @@
       <c r="C22" s="3">
         <v>0</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="9" t="s">
+      <c r="D22" s="40"/>
+      <c r="E22" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="13"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -2341,14 +2362,14 @@
       <c r="C23" s="3">
         <v>0</v>
       </c>
-      <c r="D23" s="41"/>
+      <c r="D23" s="40"/>
       <c r="E23" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="14"/>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -2360,14 +2381,14 @@
       <c r="C24" s="3">
         <v>0</v>
       </c>
-      <c r="D24" s="41"/>
+      <c r="D24" s="40"/>
       <c r="E24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F24" s="3">
         <v>0</v>
       </c>
-      <c r="G24" s="14"/>
+      <c r="G24" s="7"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -2376,17 +2397,17 @@
       <c r="B25" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="34">
+      <c r="C25" s="12">
         <v>1087616</v>
       </c>
-      <c r="D25" s="41"/>
+      <c r="D25" s="40"/>
       <c r="E25" s="3" t="s">
         <v>47</v>
       </c>
       <c r="F25" s="3">
         <v>0</v>
       </c>
-      <c r="G25" s="14"/>
+      <c r="G25" s="7"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -2395,17 +2416,17 @@
       <c r="B26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="34">
+      <c r="C26" s="12">
         <v>33226</v>
       </c>
-      <c r="D26" s="41"/>
+      <c r="D26" s="40"/>
       <c r="E26" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F26" s="3">
         <v>0</v>
       </c>
-      <c r="G26" s="14"/>
+      <c r="G26" s="7"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -2417,14 +2438,14 @@
       <c r="C27" s="3">
         <v>0</v>
       </c>
-      <c r="D27" s="41"/>
+      <c r="D27" s="40"/>
       <c r="E27" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F27" s="3">
         <v>0</v>
       </c>
-      <c r="G27" s="16"/>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -2433,15 +2454,15 @@
       <c r="B28" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="34">
+      <c r="C28" s="12">
         <v>2000</v>
       </c>
-      <c r="D28" s="41"/>
-      <c r="E28" s="35" t="s">
+      <c r="D28" s="40"/>
+      <c r="E28" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="F28" s="36"/>
-      <c r="G28" s="37"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="20"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2453,235 +2474,235 @@
       <c r="C29" s="3">
         <v>0</v>
       </c>
-      <c r="D29" s="41"/>
-      <c r="E29" s="9" t="s">
+      <c r="D29" s="40"/>
+      <c r="E29" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="F29" s="10"/>
-      <c r="G29" s="13"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="6"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="32">
+      <c r="B30" s="23"/>
+      <c r="C30" s="10">
         <v>1122842</v>
       </c>
-      <c r="D30" s="41"/>
+      <c r="D30" s="40"/>
       <c r="E30" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G30" s="14"/>
+      <c r="G30" s="7"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="44"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="41"/>
+      <c r="A31" s="42"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="40"/>
       <c r="E31" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
       </c>
-      <c r="G31" s="14"/>
+      <c r="G31" s="7"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="43"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="48"/>
-      <c r="D32" s="41"/>
+      <c r="A32" s="45"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
       </c>
-      <c r="G32" s="14"/>
+      <c r="G32" s="7"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A33" s="29"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="42"/>
+      <c r="A33" s="35"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="41"/>
       <c r="E33" s="3" t="s">
         <v>53</v>
       </c>
       <c r="F33" s="3">
         <v>0</v>
       </c>
-      <c r="G33" s="16"/>
+      <c r="G33" s="9"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="B34" s="36"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="37"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="20"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="13"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="33"/>
+      <c r="K36" s="38"/>
+      <c r="L36" s="6"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A37" s="49" t="s">
+      <c r="A37" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="B37" s="49" t="s">
+      <c r="B37" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="49" t="s">
+      <c r="C37" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="D37" s="49" t="s">
+      <c r="D37" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="49" t="s">
+      <c r="E37" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="F37" s="49" t="s">
+      <c r="F37" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="G37" s="54" t="s">
+      <c r="G37" s="61" t="s">
         <v>67</v>
       </c>
-      <c r="H37" s="55"/>
-      <c r="I37" s="49" t="s">
+      <c r="H37" s="62"/>
+      <c r="I37" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="J37" s="49" t="s">
+      <c r="J37" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="K37" s="49" t="s">
+      <c r="K37" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="L37" s="14"/>
+      <c r="L37" s="7"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B38" s="50" t="s">
+      <c r="B38" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="50" t="s">
+      <c r="C38" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="D38" s="50" t="s">
+      <c r="D38" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="E38" s="50" t="s">
+      <c r="E38" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="F38" s="50" t="s">
+      <c r="F38" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="G38" s="56"/>
-      <c r="H38" s="57"/>
-      <c r="I38" s="50" t="s">
+      <c r="G38" s="64"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="J38" s="50" t="s">
+      <c r="J38" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="K38" s="50" t="s">
+      <c r="K38" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="L38" s="14"/>
+      <c r="L38" s="7"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A39" s="50"/>
-      <c r="B39" s="50"/>
-      <c r="C39" s="50"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="50" t="s">
+      <c r="A39" s="63"/>
+      <c r="B39" s="63"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
+      <c r="E39" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="F39" s="50"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="57"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50" t="s">
+      <c r="F39" s="63"/>
+      <c r="G39" s="64"/>
+      <c r="H39" s="65"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="K39" s="50" t="s">
+      <c r="K39" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="L39" s="14"/>
+      <c r="L39" s="7"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="50"/>
-      <c r="B40" s="50"/>
-      <c r="C40" s="50"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50" t="s">
+      <c r="A40" s="63"/>
+      <c r="B40" s="63"/>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="F40" s="50"/>
-      <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="50" t="s">
+      <c r="F40" s="63"/>
+      <c r="G40" s="66"/>
+      <c r="H40" s="67"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="L40" s="14"/>
+      <c r="L40" s="7"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="50"/>
-      <c r="B41" s="50"/>
-      <c r="C41" s="50"/>
-      <c r="D41" s="50"/>
-      <c r="E41" s="50"/>
-      <c r="F41" s="50"/>
-      <c r="G41" s="60" t="s">
+      <c r="A41" s="63"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="H41" s="49" t="s">
+      <c r="H41" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="I41" s="50"/>
-      <c r="J41" s="50"/>
-      <c r="K41" s="50" t="s">
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="L41" s="14"/>
+      <c r="L41" s="7"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="51"/>
-      <c r="B42" s="51"/>
-      <c r="C42" s="51"/>
-      <c r="D42" s="51"/>
-      <c r="E42" s="51"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="61"/>
-      <c r="H42" s="51" t="s">
+      <c r="A42" s="69"/>
+      <c r="B42" s="69"/>
+      <c r="C42" s="69"/>
+      <c r="D42" s="69"/>
+      <c r="E42" s="69"/>
+      <c r="F42" s="69"/>
+      <c r="G42" s="70"/>
+      <c r="H42" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="I42" s="51"/>
-      <c r="J42" s="51"/>
-      <c r="K42" s="51"/>
-      <c r="L42" s="14"/>
+      <c r="I42" s="69"/>
+      <c r="J42" s="69"/>
+      <c r="K42" s="69"/>
+      <c r="L42" s="7"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
@@ -2693,12 +2714,12 @@
       <c r="C43" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D43" s="34">
+      <c r="D43" s="12">
         <v>10700</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
-      <c r="G43" s="34">
+      <c r="G43" s="12">
         <v>10700</v>
       </c>
       <c r="H43" s="3">
@@ -2711,7 +2732,7 @@
       <c r="K43" s="3">
         <v>0</v>
       </c>
-      <c r="L43" s="14"/>
+      <c r="L43" s="7"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
@@ -2723,12 +2744,12 @@
       <c r="C44" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D44" s="34">
+      <c r="D44" s="12">
         <v>21180</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="34">
+      <c r="G44" s="12">
         <v>21180</v>
       </c>
       <c r="H44" s="3">
@@ -2741,7 +2762,7 @@
       <c r="K44" s="3">
         <v>0</v>
       </c>
-      <c r="L44" s="14"/>
+      <c r="L44" s="7"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
@@ -2753,12 +2774,12 @@
       <c r="C45" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D45" s="34">
+      <c r="D45" s="12">
         <v>33600</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="34">
+      <c r="G45" s="12">
         <v>33600</v>
       </c>
       <c r="H45" s="3">
@@ -2771,7 +2792,7 @@
       <c r="K45" s="3">
         <v>1</v>
       </c>
-      <c r="L45" s="14"/>
+      <c r="L45" s="7"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
@@ -2783,12 +2804,12 @@
       <c r="C46" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D46" s="34">
+      <c r="D46" s="12">
         <v>8000</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
-      <c r="G46" s="34">
+      <c r="G46" s="12">
         <v>8000</v>
       </c>
       <c r="H46" s="3">
@@ -2801,7 +2822,7 @@
       <c r="K46" s="3">
         <v>2.8</v>
       </c>
-      <c r="L46" s="14"/>
+      <c r="L46" s="7"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
@@ -2813,12 +2834,12 @@
       <c r="C47" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D47" s="34">
+      <c r="D47" s="12">
         <v>9800</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="34">
+      <c r="G47" s="12">
         <v>9800</v>
       </c>
       <c r="H47" s="3">
@@ -2831,7 +2852,7 @@
       <c r="K47" s="3">
         <v>1</v>
       </c>
-      <c r="L47" s="14"/>
+      <c r="L47" s="7"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
@@ -2843,7 +2864,7 @@
       <c r="C48" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D48" s="34">
+      <c r="D48" s="12">
         <v>21354</v>
       </c>
       <c r="E48" s="2"/>
@@ -2863,7 +2884,7 @@
       <c r="K48" s="3">
         <v>0</v>
       </c>
-      <c r="L48" s="14"/>
+      <c r="L48" s="7"/>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
@@ -2875,12 +2896,12 @@
       <c r="C49" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D49" s="34">
+      <c r="D49" s="12">
         <v>18846</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
-      <c r="G49" s="34">
+      <c r="G49" s="12">
         <v>18846</v>
       </c>
       <c r="H49" s="3">
@@ -2893,7 +2914,7 @@
       <c r="K49" s="3">
         <v>1</v>
       </c>
-      <c r="L49" s="14"/>
+      <c r="L49" s="7"/>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
@@ -2905,12 +2926,12 @@
       <c r="C50" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D50" s="34">
+      <c r="D50" s="12">
         <v>23900</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
-      <c r="G50" s="34">
+      <c r="G50" s="12">
         <v>23900</v>
       </c>
       <c r="H50" s="3">
@@ -2923,7 +2944,7 @@
       <c r="K50" s="3">
         <v>1</v>
       </c>
-      <c r="L50" s="14"/>
+      <c r="L50" s="7"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
@@ -2935,12 +2956,12 @@
       <c r="C51" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D51" s="34">
+      <c r="D51" s="12">
         <v>1550</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
-      <c r="G51" s="34">
+      <c r="G51" s="12">
         <v>1550</v>
       </c>
       <c r="H51" s="3">
@@ -2953,7 +2974,7 @@
       <c r="K51" s="3">
         <v>1</v>
       </c>
-      <c r="L51" s="14"/>
+      <c r="L51" s="7"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
@@ -2965,12 +2986,12 @@
       <c r="C52" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D52" s="34">
+      <c r="D52" s="12">
         <v>36000</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
-      <c r="G52" s="34">
+      <c r="G52" s="12">
         <v>36000</v>
       </c>
       <c r="H52" s="3">
@@ -2983,7 +3004,7 @@
       <c r="K52" s="3">
         <v>1.2</v>
       </c>
-      <c r="L52" s="14"/>
+      <c r="L52" s="7"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
@@ -2995,12 +3016,12 @@
       <c r="C53" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D53" s="34">
+      <c r="D53" s="12">
         <v>16650</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
-      <c r="G53" s="34">
+      <c r="G53" s="12">
         <v>16650</v>
       </c>
       <c r="H53" s="3">
@@ -3013,7 +3034,7 @@
       <c r="K53" s="3">
         <v>3.4</v>
       </c>
-      <c r="L53" s="14"/>
+      <c r="L53" s="7"/>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
@@ -3025,12 +3046,12 @@
       <c r="C54" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D54" s="34">
+      <c r="D54" s="12">
         <v>61400</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
-      <c r="G54" s="34">
+      <c r="G54" s="12">
         <v>61400</v>
       </c>
       <c r="H54" s="3">
@@ -3043,7 +3064,7 @@
       <c r="K54" s="3">
         <v>1.2</v>
       </c>
-      <c r="L54" s="14"/>
+      <c r="L54" s="7"/>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
@@ -3055,12 +3076,12 @@
       <c r="C55" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D55" s="34">
+      <c r="D55" s="12">
         <v>23500</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="34">
+      <c r="G55" s="12">
         <v>23500</v>
       </c>
       <c r="H55" s="3">
@@ -3073,7 +3094,7 @@
       <c r="K55" s="3">
         <v>1.2</v>
       </c>
-      <c r="L55" s="14"/>
+      <c r="L55" s="7"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
@@ -3085,12 +3106,12 @@
       <c r="C56" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D56" s="34">
+      <c r="D56" s="12">
         <v>17900</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="34">
+      <c r="G56" s="12">
         <v>17900</v>
       </c>
       <c r="H56" s="3">
@@ -3103,7 +3124,7 @@
       <c r="K56" s="3">
         <v>1.2</v>
       </c>
-      <c r="L56" s="14"/>
+      <c r="L56" s="7"/>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -3115,12 +3136,12 @@
       <c r="C57" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D57" s="34">
+      <c r="D57" s="12">
         <v>18000</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
-      <c r="G57" s="34">
+      <c r="G57" s="12">
         <v>18000</v>
       </c>
       <c r="H57" s="3">
@@ -3133,7 +3154,7 @@
       <c r="K57" s="3">
         <v>1.2</v>
       </c>
-      <c r="L57" s="14"/>
+      <c r="L57" s="7"/>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
@@ -3145,12 +3166,12 @@
       <c r="C58" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D58" s="34">
+      <c r="D58" s="12">
         <v>8200</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
-      <c r="G58" s="34">
+      <c r="G58" s="12">
         <v>8200</v>
       </c>
       <c r="H58" s="3">
@@ -3163,7 +3184,7 @@
       <c r="K58" s="3">
         <v>1.2</v>
       </c>
-      <c r="L58" s="14"/>
+      <c r="L58" s="7"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
@@ -3175,12 +3196,12 @@
       <c r="C59" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D59" s="34">
+      <c r="D59" s="12">
         <v>14000</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
-      <c r="G59" s="34">
+      <c r="G59" s="12">
         <v>14000</v>
       </c>
       <c r="H59" s="3">
@@ -3193,7 +3214,7 @@
       <c r="K59" s="3">
         <v>1.2</v>
       </c>
-      <c r="L59" s="14"/>
+      <c r="L59" s="7"/>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
@@ -3205,12 +3226,12 @@
       <c r="C60" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D60" s="34">
+      <c r="D60" s="12">
         <v>6000</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
-      <c r="G60" s="34">
+      <c r="G60" s="12">
         <v>6000</v>
       </c>
       <c r="H60" s="3">
@@ -3223,7 +3244,7 @@
       <c r="K60" s="3">
         <v>1.2</v>
       </c>
-      <c r="L60" s="14"/>
+      <c r="L60" s="7"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
@@ -3235,12 +3256,12 @@
       <c r="C61" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D61" s="34">
+      <c r="D61" s="12">
         <v>4500</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
-      <c r="G61" s="34">
+      <c r="G61" s="12">
         <v>4500</v>
       </c>
       <c r="H61" s="3">
@@ -3253,7 +3274,7 @@
       <c r="K61" s="3">
         <v>1.2</v>
       </c>
-      <c r="L61" s="14"/>
+      <c r="L61" s="7"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
@@ -3265,12 +3286,12 @@
       <c r="C62" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D62" s="34">
+      <c r="D62" s="12">
         <v>85000</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
-      <c r="G62" s="34">
+      <c r="G62" s="12">
         <v>85000</v>
       </c>
       <c r="H62" s="3">
@@ -3283,7 +3304,7 @@
       <c r="K62" s="3">
         <v>1.2</v>
       </c>
-      <c r="L62" s="14"/>
+      <c r="L62" s="7"/>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
@@ -3313,7 +3334,7 @@
       <c r="K63" s="3">
         <v>1.2</v>
       </c>
-      <c r="L63" s="14"/>
+      <c r="L63" s="7"/>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
@@ -3325,12 +3346,12 @@
       <c r="C64" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D64" s="34">
+      <c r="D64" s="12">
         <v>15700</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
-      <c r="G64" s="34">
+      <c r="G64" s="12">
         <v>15700</v>
       </c>
       <c r="H64" s="3">
@@ -3343,7 +3364,7 @@
       <c r="K64" s="3">
         <v>0.1</v>
       </c>
-      <c r="L64" s="14"/>
+      <c r="L64" s="7"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
@@ -3355,12 +3376,12 @@
       <c r="C65" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D65" s="34">
+      <c r="D65" s="12">
         <v>29600</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
-      <c r="G65" s="34">
+      <c r="G65" s="12">
         <v>29600</v>
       </c>
       <c r="H65" s="3">
@@ -3373,7 +3394,7 @@
       <c r="K65" s="3">
         <v>1.2</v>
       </c>
-      <c r="L65" s="14"/>
+      <c r="L65" s="7"/>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
@@ -3385,12 +3406,12 @@
       <c r="C66" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D66" s="34">
+      <c r="D66" s="12">
         <v>6900</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
-      <c r="G66" s="34">
+      <c r="G66" s="12">
         <v>6900</v>
       </c>
       <c r="H66" s="3">
@@ -3403,7 +3424,7 @@
       <c r="K66" s="3">
         <v>1.2</v>
       </c>
-      <c r="L66" s="14"/>
+      <c r="L66" s="7"/>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
@@ -3415,12 +3436,12 @@
       <c r="C67" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D67" s="34">
+      <c r="D67" s="12">
         <v>21690</v>
       </c>
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
-      <c r="G67" s="34">
+      <c r="G67" s="12">
         <v>21690</v>
       </c>
       <c r="H67" s="3">
@@ -3433,7 +3454,7 @@
       <c r="K67" s="3">
         <v>1.2</v>
       </c>
-      <c r="L67" s="14"/>
+      <c r="L67" s="7"/>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
@@ -3445,12 +3466,12 @@
       <c r="C68" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D68" s="34">
+      <c r="D68" s="12">
         <v>12900</v>
       </c>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
-      <c r="G68" s="34">
+      <c r="G68" s="12">
         <v>12900</v>
       </c>
       <c r="H68" s="3">
@@ -3463,7 +3484,7 @@
       <c r="K68" s="3">
         <v>1.2</v>
       </c>
-      <c r="L68" s="14"/>
+      <c r="L68" s="7"/>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
@@ -3475,12 +3496,12 @@
       <c r="C69" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D69" s="34">
+      <c r="D69" s="12">
         <v>21200</v>
       </c>
       <c r="E69" s="2"/>
       <c r="F69" s="2"/>
-      <c r="G69" s="34">
+      <c r="G69" s="12">
         <v>21200</v>
       </c>
       <c r="H69" s="3">
@@ -3493,7 +3514,7 @@
       <c r="K69" s="3">
         <v>1.2</v>
       </c>
-      <c r="L69" s="14"/>
+      <c r="L69" s="7"/>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
@@ -3505,12 +3526,12 @@
       <c r="C70" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D70" s="34">
+      <c r="D70" s="12">
         <v>19800</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" s="2"/>
-      <c r="G70" s="34">
+      <c r="G70" s="12">
         <v>19800</v>
       </c>
       <c r="H70" s="3">
@@ -3523,7 +3544,7 @@
       <c r="K70" s="3">
         <v>1.2</v>
       </c>
-      <c r="L70" s="14"/>
+      <c r="L70" s="7"/>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
@@ -3535,12 +3556,12 @@
       <c r="C71" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D71" s="34">
+      <c r="D71" s="12">
         <v>133000</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" s="2"/>
-      <c r="G71" s="34">
+      <c r="G71" s="12">
         <v>133000</v>
       </c>
       <c r="H71" s="3">
@@ -3553,7 +3574,7 @@
       <c r="K71" s="3">
         <v>1.2</v>
       </c>
-      <c r="L71" s="14"/>
+      <c r="L71" s="7"/>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
@@ -3565,12 +3586,12 @@
       <c r="C72" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D72" s="34">
+      <c r="D72" s="12">
         <v>74600</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
-      <c r="G72" s="34">
+      <c r="G72" s="12">
         <v>74600</v>
       </c>
       <c r="H72" s="3">
@@ -3583,7 +3604,7 @@
       <c r="K72" s="3">
         <v>1.2</v>
       </c>
-      <c r="L72" s="14"/>
+      <c r="L72" s="7"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
@@ -3595,12 +3616,12 @@
       <c r="C73" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D73" s="34">
+      <c r="D73" s="12">
         <v>2900</v>
       </c>
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
-      <c r="G73" s="34">
+      <c r="G73" s="12">
         <v>2900</v>
       </c>
       <c r="H73" s="3">
@@ -3613,7 +3634,7 @@
       <c r="K73" s="3">
         <v>3.4</v>
       </c>
-      <c r="L73" s="14"/>
+      <c r="L73" s="7"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
@@ -3625,12 +3646,12 @@
       <c r="C74" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D74" s="34">
+      <c r="D74" s="12">
         <v>1800</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
-      <c r="G74" s="34">
+      <c r="G74" s="12">
         <v>1800</v>
       </c>
       <c r="H74" s="3">
@@ -3643,7 +3664,7 @@
       <c r="K74" s="3">
         <v>3.4</v>
       </c>
-      <c r="L74" s="14"/>
+      <c r="L74" s="7"/>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
@@ -3655,12 +3676,12 @@
       <c r="C75" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D75" s="34">
+      <c r="D75" s="12">
         <v>11900</v>
       </c>
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
-      <c r="G75" s="34">
+      <c r="G75" s="12">
         <v>11900</v>
       </c>
       <c r="H75" s="3">
@@ -3673,7 +3694,7 @@
       <c r="K75" s="3">
         <v>1.2</v>
       </c>
-      <c r="L75" s="14"/>
+      <c r="L75" s="7"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
@@ -3685,12 +3706,12 @@
       <c r="C76" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D76" s="34">
+      <c r="D76" s="12">
         <v>11500</v>
       </c>
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
-      <c r="G76" s="34">
+      <c r="G76" s="12">
         <v>11500</v>
       </c>
       <c r="H76" s="3">
@@ -3703,7 +3724,7 @@
       <c r="K76" s="3">
         <v>1.2</v>
       </c>
-      <c r="L76" s="14"/>
+      <c r="L76" s="7"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
@@ -3715,12 +3736,12 @@
       <c r="C77" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D77" s="34">
+      <c r="D77" s="12">
         <v>199000</v>
       </c>
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="34">
+      <c r="G77" s="12">
         <v>199000</v>
       </c>
       <c r="H77" s="3">
@@ -3733,7 +3754,7 @@
       <c r="K77" s="3">
         <v>1.2</v>
       </c>
-      <c r="L77" s="14"/>
+      <c r="L77" s="7"/>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
@@ -3745,12 +3766,12 @@
       <c r="C78" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D78" s="34">
+      <c r="D78" s="12">
         <v>106000</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="34">
+      <c r="G78" s="12">
         <v>106000</v>
       </c>
       <c r="H78" s="3">
@@ -3763,73 +3784,73 @@
       <c r="K78" s="3">
         <v>1.2</v>
       </c>
-      <c r="L78" s="14"/>
+      <c r="L78" s="7"/>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A79" s="5" t="s">
+      <c r="A79" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="B79" s="39"/>
-      <c r="C79" s="39"/>
-      <c r="D79" s="6"/>
+      <c r="B79" s="22"/>
+      <c r="C79" s="22"/>
+      <c r="D79" s="23"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="52">
+      <c r="G79" s="16">
         <v>31880</v>
       </c>
-      <c r="H79" s="53">
+      <c r="H79" s="17">
         <v>0</v>
       </c>
       <c r="I79" s="2"/>
-      <c r="J79" s="53">
+      <c r="J79" s="17">
         <v>0</v>
       </c>
       <c r="K79" s="2"/>
-      <c r="L79" s="14"/>
+      <c r="L79" s="7"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A80" s="5" t="s">
+      <c r="A80" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B80" s="39"/>
-      <c r="C80" s="39"/>
-      <c r="D80" s="6"/>
+      <c r="B80" s="22"/>
+      <c r="C80" s="22"/>
+      <c r="D80" s="23"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="52">
+      <c r="G80" s="16">
         <v>1055736</v>
       </c>
-      <c r="H80" s="53">
+      <c r="H80" s="17">
         <v>0</v>
       </c>
       <c r="I80" s="2"/>
-      <c r="J80" s="53">
+      <c r="J80" s="17">
         <v>0</v>
       </c>
       <c r="K80" s="2"/>
-      <c r="L80" s="14"/>
+      <c r="L80" s="7"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="5" t="s">
+      <c r="A81" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="B81" s="39"/>
-      <c r="C81" s="39"/>
-      <c r="D81" s="6"/>
+      <c r="B81" s="22"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="23"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="52">
+      <c r="G81" s="16">
         <v>1087616</v>
       </c>
-      <c r="H81" s="53">
+      <c r="H81" s="17">
         <v>0</v>
       </c>
       <c r="I81" s="2"/>
-      <c r="J81" s="53">
+      <c r="J81" s="17">
         <v>0</v>
       </c>
       <c r="K81" s="2"/>
-      <c r="L81" s="14"/>
+      <c r="L81" s="7"/>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
@@ -3846,7 +3867,7 @@
       </c>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="34">
+      <c r="G82" s="12">
         <v>33167</v>
       </c>
       <c r="H82" s="3">
@@ -3859,51 +3880,51 @@
       <c r="K82" s="3">
         <v>3.4</v>
       </c>
-      <c r="L82" s="14"/>
+      <c r="L82" s="7"/>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A83" s="5" t="s">
+      <c r="A83" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="B83" s="39"/>
-      <c r="C83" s="39"/>
-      <c r="D83" s="6"/>
+      <c r="B83" s="22"/>
+      <c r="C83" s="22"/>
+      <c r="D83" s="23"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="52">
+      <c r="G83" s="16">
         <v>33167</v>
       </c>
-      <c r="H83" s="53">
+      <c r="H83" s="17">
         <v>59</v>
       </c>
       <c r="I83" s="2"/>
-      <c r="J83" s="53">
+      <c r="J83" s="17">
         <v>0</v>
       </c>
       <c r="K83" s="2"/>
-      <c r="L83" s="14"/>
+      <c r="L83" s="7"/>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B84" s="39"/>
-      <c r="C84" s="39"/>
-      <c r="D84" s="6"/>
+      <c r="B84" s="22"/>
+      <c r="C84" s="22"/>
+      <c r="D84" s="23"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="52">
+      <c r="G84" s="16">
         <v>33167</v>
       </c>
-      <c r="H84" s="53">
+      <c r="H84" s="17">
         <v>59</v>
       </c>
       <c r="I84" s="2"/>
-      <c r="J84" s="53">
+      <c r="J84" s="17">
         <v>0</v>
       </c>
       <c r="K84" s="2"/>
-      <c r="L84" s="14"/>
+      <c r="L84" s="7"/>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
@@ -3913,12 +3934,12 @@
       <c r="C85" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="D85" s="34">
+      <c r="D85" s="12">
         <v>2000</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="34">
+      <c r="G85" s="12">
         <v>2000</v>
       </c>
       <c r="H85" s="3">
@@ -3931,215 +3952,215 @@
       <c r="K85" s="3">
         <v>0</v>
       </c>
-      <c r="L85" s="14"/>
+      <c r="L85" s="7"/>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A86" s="5" t="s">
+      <c r="A86" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B86" s="39"/>
-      <c r="C86" s="39"/>
-      <c r="D86" s="6"/>
+      <c r="B86" s="22"/>
+      <c r="C86" s="22"/>
+      <c r="D86" s="23"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="52">
+      <c r="G86" s="16">
         <v>2000</v>
       </c>
-      <c r="H86" s="53">
+      <c r="H86" s="17">
         <v>0</v>
       </c>
       <c r="I86" s="2"/>
-      <c r="J86" s="53">
+      <c r="J86" s="17">
         <v>0</v>
       </c>
       <c r="K86" s="2"/>
-      <c r="L86" s="14"/>
+      <c r="L86" s="7"/>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A87" s="5" t="s">
+      <c r="A87" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="B87" s="39"/>
-      <c r="C87" s="39"/>
-      <c r="D87" s="6"/>
+      <c r="B87" s="22"/>
+      <c r="C87" s="22"/>
+      <c r="D87" s="23"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="52">
+      <c r="G87" s="16">
         <v>1122783</v>
       </c>
-      <c r="H87" s="53">
+      <c r="H87" s="17">
         <v>59</v>
       </c>
       <c r="I87" s="2"/>
-      <c r="J87" s="53">
+      <c r="J87" s="17">
         <v>0</v>
       </c>
       <c r="K87" s="2"/>
-      <c r="L87" s="14"/>
+      <c r="L87" s="7"/>
     </row>
     <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="5" t="s">
+      <c r="A88" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B88" s="39"/>
-      <c r="C88" s="39"/>
-      <c r="D88" s="39"/>
-      <c r="E88" s="39"/>
-      <c r="F88" s="39"/>
-      <c r="G88" s="39"/>
-      <c r="H88" s="39"/>
-      <c r="I88" s="39"/>
-      <c r="J88" s="39"/>
-      <c r="K88" s="6"/>
-      <c r="L88" s="14"/>
+      <c r="B88" s="22"/>
+      <c r="C88" s="22"/>
+      <c r="D88" s="22"/>
+      <c r="E88" s="22"/>
+      <c r="F88" s="22"/>
+      <c r="G88" s="22"/>
+      <c r="H88" s="22"/>
+      <c r="I88" s="22"/>
+      <c r="J88" s="22"/>
+      <c r="K88" s="23"/>
+      <c r="L88" s="7"/>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A89" s="7"/>
-      <c r="B89" s="38"/>
-      <c r="C89" s="38"/>
-      <c r="D89" s="38"/>
-      <c r="E89" s="38"/>
-      <c r="F89" s="38"/>
-      <c r="G89" s="38"/>
-      <c r="H89" s="38"/>
-      <c r="I89" s="38"/>
-      <c r="J89" s="38"/>
-      <c r="K89" s="8"/>
-      <c r="L89" s="14"/>
+      <c r="A89" s="24"/>
+      <c r="B89" s="25"/>
+      <c r="C89" s="25"/>
+      <c r="D89" s="25"/>
+      <c r="E89" s="25"/>
+      <c r="F89" s="25"/>
+      <c r="G89" s="25"/>
+      <c r="H89" s="25"/>
+      <c r="I89" s="25"/>
+      <c r="J89" s="25"/>
+      <c r="K89" s="26"/>
+      <c r="L89" s="7"/>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A90" s="9" t="s">
+      <c r="A90" s="32" t="s">
         <v>140</v>
       </c>
-      <c r="B90" s="10"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="10"/>
-      <c r="E90" s="10"/>
-      <c r="F90" s="10"/>
-      <c r="G90" s="10"/>
-      <c r="H90" s="10"/>
-      <c r="I90" s="12"/>
-      <c r="J90" s="12"/>
-      <c r="K90" s="13"/>
-      <c r="L90" s="14"/>
+      <c r="B90" s="33"/>
+      <c r="C90" s="33"/>
+      <c r="D90" s="33"/>
+      <c r="E90" s="33"/>
+      <c r="F90" s="33"/>
+      <c r="G90" s="33"/>
+      <c r="H90" s="33"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="K90" s="6"/>
+      <c r="L90" s="7"/>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A91" s="60" t="s">
+      <c r="A91" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="B91" s="60" t="s">
+      <c r="B91" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="C91" s="60" t="s">
+      <c r="C91" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="D91" s="60" t="s">
+      <c r="D91" s="30" t="s">
         <v>144</v>
       </c>
-      <c r="E91" s="60" t="s">
+      <c r="E91" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="F91" s="5" t="s">
+      <c r="F91" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="G91" s="6"/>
-      <c r="H91" s="49" t="s">
+      <c r="G91" s="23"/>
+      <c r="H91" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="K91" s="14"/>
-      <c r="L91" s="14"/>
+      <c r="K91" s="7"/>
+      <c r="L91" s="7"/>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A92" s="62"/>
-      <c r="B92" s="62"/>
-      <c r="C92" s="62"/>
-      <c r="D92" s="62"/>
-      <c r="E92" s="62"/>
-      <c r="F92" s="60" t="s">
+      <c r="A92" s="34"/>
+      <c r="B92" s="34"/>
+      <c r="C92" s="34"/>
+      <c r="D92" s="34"/>
+      <c r="E92" s="34"/>
+      <c r="F92" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="G92" s="49" t="s">
+      <c r="G92" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="H92" s="50" t="s">
+      <c r="H92" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="K92" s="14"/>
-      <c r="L92" s="14"/>
+      <c r="K92" s="7"/>
+      <c r="L92" s="7"/>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A93" s="61"/>
-      <c r="B93" s="61"/>
-      <c r="C93" s="61"/>
-      <c r="D93" s="61"/>
-      <c r="E93" s="61"/>
-      <c r="F93" s="61"/>
-      <c r="G93" s="51" t="s">
+      <c r="A93" s="31"/>
+      <c r="B93" s="31"/>
+      <c r="C93" s="31"/>
+      <c r="D93" s="31"/>
+      <c r="E93" s="31"/>
+      <c r="F93" s="31"/>
+      <c r="G93" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="H93" s="51"/>
-      <c r="K93" s="14"/>
-      <c r="L93" s="14"/>
+      <c r="H93" s="15"/>
+      <c r="K93" s="7"/>
+      <c r="L93" s="7"/>
     </row>
     <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B94" s="39"/>
-      <c r="C94" s="39"/>
-      <c r="D94" s="39"/>
-      <c r="E94" s="6"/>
-      <c r="F94" s="53"/>
-      <c r="G94" s="53"/>
-      <c r="H94" s="53"/>
-      <c r="K94" s="14"/>
-      <c r="L94" s="14"/>
+      <c r="B94" s="22"/>
+      <c r="C94" s="22"/>
+      <c r="D94" s="22"/>
+      <c r="E94" s="23"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="17"/>
+      <c r="H94" s="17"/>
+      <c r="K94" s="7"/>
+      <c r="L94" s="7"/>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A95" s="5" t="s">
+      <c r="A95" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="B95" s="39"/>
-      <c r="C95" s="39"/>
-      <c r="D95" s="39"/>
-      <c r="E95" s="39"/>
-      <c r="F95" s="39"/>
-      <c r="G95" s="39"/>
-      <c r="H95" s="6"/>
-      <c r="I95" s="15"/>
-      <c r="J95" s="15"/>
-      <c r="K95" s="16"/>
-      <c r="L95" s="14"/>
+      <c r="B95" s="22"/>
+      <c r="C95" s="22"/>
+      <c r="D95" s="22"/>
+      <c r="E95" s="22"/>
+      <c r="F95" s="22"/>
+      <c r="G95" s="22"/>
+      <c r="H95" s="23"/>
+      <c r="I95" s="8"/>
+      <c r="J95" s="8"/>
+      <c r="K95" s="9"/>
+      <c r="L95" s="7"/>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A96" s="7"/>
-      <c r="B96" s="38"/>
-      <c r="C96" s="38"/>
-      <c r="D96" s="38"/>
-      <c r="E96" s="38"/>
-      <c r="F96" s="38"/>
-      <c r="G96" s="38"/>
-      <c r="H96" s="38"/>
-      <c r="I96" s="38"/>
-      <c r="J96" s="38"/>
-      <c r="K96" s="8"/>
-      <c r="L96" s="14"/>
+      <c r="A96" s="24"/>
+      <c r="B96" s="25"/>
+      <c r="C96" s="25"/>
+      <c r="D96" s="25"/>
+      <c r="E96" s="25"/>
+      <c r="F96" s="25"/>
+      <c r="G96" s="25"/>
+      <c r="H96" s="25"/>
+      <c r="I96" s="25"/>
+      <c r="J96" s="25"/>
+      <c r="K96" s="26"/>
+      <c r="L96" s="7"/>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A97" s="9" t="s">
+      <c r="A97" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B97" s="10"/>
-      <c r="C97" s="10"/>
-      <c r="D97" s="10"/>
-      <c r="E97" s="10"/>
-      <c r="F97" s="10"/>
-      <c r="G97" s="10"/>
-      <c r="H97" s="10"/>
-      <c r="I97" s="10"/>
-      <c r="J97" s="12"/>
-      <c r="K97" s="13"/>
-      <c r="L97" s="63"/>
+      <c r="B97" s="33"/>
+      <c r="C97" s="33"/>
+      <c r="D97" s="33"/>
+      <c r="E97" s="33"/>
+      <c r="F97" s="33"/>
+      <c r="G97" s="33"/>
+      <c r="H97" s="33"/>
+      <c r="I97" s="33"/>
+      <c r="J97" s="5"/>
+      <c r="K97" s="6"/>
+      <c r="L97" s="27"/>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
@@ -4169,83 +4190,83 @@
       <c r="I98" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K98" s="14"/>
-      <c r="L98" s="64"/>
+      <c r="K98" s="7"/>
+      <c r="L98" s="28"/>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A99" s="5" t="s">
+      <c r="A99" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="B99" s="39"/>
-      <c r="C99" s="39"/>
-      <c r="D99" s="39"/>
-      <c r="E99" s="39"/>
-      <c r="F99" s="39"/>
-      <c r="G99" s="39"/>
-      <c r="H99" s="39"/>
-      <c r="I99" s="6"/>
-      <c r="J99" s="15"/>
-      <c r="K99" s="16"/>
-      <c r="L99" s="65"/>
+      <c r="B99" s="22"/>
+      <c r="C99" s="22"/>
+      <c r="D99" s="22"/>
+      <c r="E99" s="22"/>
+      <c r="F99" s="22"/>
+      <c r="G99" s="22"/>
+      <c r="H99" s="22"/>
+      <c r="I99" s="23"/>
+      <c r="J99" s="8"/>
+      <c r="K99" s="9"/>
+      <c r="L99" s="29"/>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A100" s="7"/>
-      <c r="B100" s="38"/>
-      <c r="C100" s="38"/>
-      <c r="D100" s="38"/>
-      <c r="E100" s="38"/>
-      <c r="F100" s="38"/>
-      <c r="G100" s="38"/>
-      <c r="H100" s="38"/>
-      <c r="I100" s="38"/>
-      <c r="J100" s="38"/>
-      <c r="K100" s="8"/>
-      <c r="L100" s="14"/>
+      <c r="A100" s="24"/>
+      <c r="B100" s="25"/>
+      <c r="C100" s="25"/>
+      <c r="D100" s="25"/>
+      <c r="E100" s="25"/>
+      <c r="F100" s="25"/>
+      <c r="G100" s="25"/>
+      <c r="H100" s="25"/>
+      <c r="I100" s="25"/>
+      <c r="J100" s="25"/>
+      <c r="K100" s="26"/>
+      <c r="L100" s="7"/>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A101" s="9" t="s">
+      <c r="A101" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="B101" s="10"/>
-      <c r="C101" s="10"/>
-      <c r="D101" s="10"/>
-      <c r="E101" s="10"/>
-      <c r="F101" s="10"/>
-      <c r="G101" s="10"/>
-      <c r="H101" s="10"/>
-      <c r="I101" s="12"/>
-      <c r="J101" s="12"/>
-      <c r="K101" s="13"/>
-      <c r="L101" s="14"/>
+      <c r="B101" s="33"/>
+      <c r="C101" s="33"/>
+      <c r="D101" s="33"/>
+      <c r="E101" s="33"/>
+      <c r="F101" s="33"/>
+      <c r="G101" s="33"/>
+      <c r="H101" s="33"/>
+      <c r="I101" s="5"/>
+      <c r="J101" s="5"/>
+      <c r="K101" s="6"/>
+      <c r="L101" s="7"/>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A102" s="60" t="s">
+      <c r="A102" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="B102" s="60" t="s">
+      <c r="B102" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="C102" s="60" t="s">
+      <c r="C102" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D102" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="E102" s="6"/>
-      <c r="F102" s="5" t="s">
+      <c r="E102" s="23"/>
+      <c r="F102" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="G102" s="6"/>
-      <c r="H102" s="60" t="s">
+      <c r="G102" s="23"/>
+      <c r="H102" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="K102" s="14"/>
-      <c r="L102" s="14"/>
+      <c r="K102" s="7"/>
+      <c r="L102" s="7"/>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A103" s="61"/>
-      <c r="B103" s="61"/>
-      <c r="C103" s="61"/>
+      <c r="A103" s="31"/>
+      <c r="B103" s="31"/>
+      <c r="C103" s="31"/>
       <c r="D103" s="1" t="s">
         <v>78</v>
       </c>
@@ -4258,73 +4279,73 @@
       <c r="G103" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="H103" s="61"/>
-      <c r="K103" s="14"/>
-      <c r="L103" s="14"/>
+      <c r="H103" s="31"/>
+      <c r="K103" s="7"/>
+      <c r="L103" s="7"/>
     </row>
     <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="5" t="s">
+      <c r="A104" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B104" s="39"/>
-      <c r="C104" s="39"/>
-      <c r="D104" s="39"/>
-      <c r="E104" s="6"/>
-      <c r="F104" s="53">
-        <v>0</v>
-      </c>
-      <c r="G104" s="53">
+      <c r="B104" s="22"/>
+      <c r="C104" s="22"/>
+      <c r="D104" s="22"/>
+      <c r="E104" s="23"/>
+      <c r="F104" s="17">
+        <v>0</v>
+      </c>
+      <c r="G104" s="17">
         <v>0</v>
       </c>
       <c r="H104" s="3"/>
-      <c r="K104" s="14"/>
-      <c r="L104" s="14"/>
+      <c r="K104" s="7"/>
+      <c r="L104" s="7"/>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A105" s="5" t="s">
+      <c r="A105" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="B105" s="39"/>
-      <c r="C105" s="39"/>
-      <c r="D105" s="39"/>
-      <c r="E105" s="39"/>
-      <c r="F105" s="39"/>
-      <c r="G105" s="39"/>
-      <c r="H105" s="6"/>
-      <c r="I105" s="15"/>
-      <c r="J105" s="15"/>
-      <c r="K105" s="16"/>
-      <c r="L105" s="14"/>
+      <c r="B105" s="22"/>
+      <c r="C105" s="22"/>
+      <c r="D105" s="22"/>
+      <c r="E105" s="22"/>
+      <c r="F105" s="22"/>
+      <c r="G105" s="22"/>
+      <c r="H105" s="23"/>
+      <c r="I105" s="8"/>
+      <c r="J105" s="8"/>
+      <c r="K105" s="9"/>
+      <c r="L105" s="7"/>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A106" s="7"/>
-      <c r="B106" s="38"/>
-      <c r="C106" s="38"/>
-      <c r="D106" s="38"/>
-      <c r="E106" s="38"/>
-      <c r="F106" s="38"/>
-      <c r="G106" s="38"/>
-      <c r="H106" s="38"/>
-      <c r="I106" s="38"/>
-      <c r="J106" s="38"/>
-      <c r="K106" s="8"/>
-      <c r="L106" s="14"/>
+      <c r="A106" s="24"/>
+      <c r="B106" s="25"/>
+      <c r="C106" s="25"/>
+      <c r="D106" s="25"/>
+      <c r="E106" s="25"/>
+      <c r="F106" s="25"/>
+      <c r="G106" s="25"/>
+      <c r="H106" s="25"/>
+      <c r="I106" s="25"/>
+      <c r="J106" s="25"/>
+      <c r="K106" s="26"/>
+      <c r="L106" s="7"/>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A107" s="9" t="s">
+      <c r="A107" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="B107" s="10"/>
-      <c r="C107" s="10"/>
-      <c r="D107" s="10"/>
-      <c r="E107" s="10"/>
-      <c r="F107" s="10"/>
-      <c r="G107" s="10"/>
-      <c r="H107" s="10"/>
-      <c r="I107" s="12"/>
-      <c r="J107" s="12"/>
-      <c r="K107" s="13"/>
-      <c r="L107" s="63"/>
+      <c r="B107" s="33"/>
+      <c r="C107" s="33"/>
+      <c r="D107" s="33"/>
+      <c r="E107" s="33"/>
+      <c r="F107" s="33"/>
+      <c r="G107" s="33"/>
+      <c r="H107" s="33"/>
+      <c r="I107" s="5"/>
+      <c r="J107" s="5"/>
+      <c r="K107" s="6"/>
+      <c r="L107" s="27"/>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
@@ -4336,54 +4357,115 @@
       <c r="C108" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D108" s="5" t="s">
+      <c r="D108" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E108" s="6"/>
-      <c r="F108" s="5" t="s">
+      <c r="E108" s="23"/>
+      <c r="F108" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="G108" s="6"/>
+      <c r="G108" s="23"/>
       <c r="H108" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="K108" s="14"/>
-      <c r="L108" s="64"/>
+      <c r="K108" s="7"/>
+      <c r="L108" s="28"/>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A109" s="5" t="s">
+      <c r="A109" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="B109" s="39"/>
-      <c r="C109" s="39"/>
-      <c r="D109" s="39"/>
-      <c r="E109" s="39"/>
-      <c r="F109" s="39"/>
-      <c r="G109" s="39"/>
-      <c r="H109" s="6"/>
-      <c r="I109" s="15"/>
-      <c r="J109" s="15"/>
-      <c r="K109" s="16"/>
-      <c r="L109" s="65"/>
+      <c r="B109" s="22"/>
+      <c r="C109" s="22"/>
+      <c r="D109" s="22"/>
+      <c r="E109" s="22"/>
+      <c r="F109" s="22"/>
+      <c r="G109" s="22"/>
+      <c r="H109" s="23"/>
+      <c r="I109" s="8"/>
+      <c r="J109" s="8"/>
+      <c r="K109" s="9"/>
+      <c r="L109" s="29"/>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A110" s="35" t="s">
+      <c r="A110" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B110" s="36"/>
-      <c r="C110" s="36"/>
-      <c r="D110" s="36"/>
-      <c r="E110" s="36"/>
-      <c r="F110" s="36"/>
-      <c r="G110" s="36"/>
-      <c r="H110" s="36"/>
-      <c r="I110" s="36"/>
-      <c r="J110" s="36"/>
-      <c r="K110" s="37"/>
+      <c r="B110" s="19"/>
+      <c r="C110" s="19"/>
+      <c r="D110" s="19"/>
+      <c r="E110" s="19"/>
+      <c r="F110" s="19"/>
+      <c r="G110" s="19"/>
+      <c r="H110" s="19"/>
+      <c r="I110" s="19"/>
+      <c r="J110" s="19"/>
+      <c r="K110" s="20"/>
       <c r="L110" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="77">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:D33"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="G37:H40"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A81:D81"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A84:D84"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A88:K88"/>
+    <mergeCell ref="A90:H90"/>
+    <mergeCell ref="A91:A93"/>
+    <mergeCell ref="B91:B93"/>
+    <mergeCell ref="C91:C93"/>
+    <mergeCell ref="D91:D93"/>
+    <mergeCell ref="E91:E93"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="F92:F93"/>
+    <mergeCell ref="A97:I97"/>
+    <mergeCell ref="A99:I99"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A102:A103"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="C102:C103"/>
+    <mergeCell ref="D102:E102"/>
+    <mergeCell ref="F102:G102"/>
     <mergeCell ref="A110:K110"/>
     <mergeCell ref="A109:H109"/>
     <mergeCell ref="A89:K89"/>
@@ -4400,67 +4482,6 @@
     <mergeCell ref="F108:G108"/>
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="A95:H95"/>
-    <mergeCell ref="A97:I97"/>
-    <mergeCell ref="A99:I99"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A102:A103"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="C102:C103"/>
-    <mergeCell ref="D102:E102"/>
-    <mergeCell ref="F102:G102"/>
-    <mergeCell ref="A88:K88"/>
-    <mergeCell ref="A90:H90"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="B91:B93"/>
-    <mergeCell ref="C91:C93"/>
-    <mergeCell ref="D91:D93"/>
-    <mergeCell ref="E91:E93"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="F92:F93"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A81:D81"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A84:D84"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="G37:H40"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:D33"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>